<commit_message>
feat(finance): reconcile cash on hand, integrate lathe charges in job profit, and polish PDF export
- Add migration 0015 for fleet invoices and cash ledger postings
- Add migration 0016 reconciling cash on hand to Rs. 50,796.00 and handling reversed transaction
- Fix accounts popup scrolling and layout in Accounts section
- Integrate lathe charges alongside crimping and welding across invoices, unpaid labour list, and Job Profit Analysis
- Support lathe charges in Excel and PDF job profit exports with mirrored market rates
- Remove redundant Invoice Total column from Job Profit Analysis PDF export for improved A4 landscape layout
- Update hydraulic.db with verified migrations and balanced ledger
</commit_message>
<xml_diff>
--- a/June_Invoice_Profit_Analysis.xlsx
+++ b/June_Invoice_Profit_Analysis.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\hy 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DABD057A-DA4F-4FE9-81E3-2CB0126FD0E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52536AFA-9814-40AD-A000-1C7345906953}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="June Summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -514,9 +514,6 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -564,6 +561,9 @@
     <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="4" fontId="6" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1702,167 +1702,167 @@
       <c r="M29" s="5"/>
     </row>
     <row r="33" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="8" t="s">
+      <c r="A33" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
+      <c r="B33" s="26"/>
+      <c r="C33" s="26"/>
+      <c r="D33" s="26"/>
+      <c r="E33" s="26"/>
     </row>
     <row r="34" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="10" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="str">
+      <c r="A35" s="11" t="str">
         <f>A2</f>
         <v>INV/2026/06/001</v>
       </c>
-      <c r="B35" s="13">
+      <c r="B35" s="12">
         <f>G2</f>
         <v>10881.97</v>
       </c>
-      <c r="C35" s="14">
+      <c r="C35" s="13">
         <f>L2</f>
         <v>20570.87</v>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="14">
         <f>C35-B35</f>
         <v>9688.9</v>
       </c>
-      <c r="E35" s="16">
+      <c r="E35" s="15">
         <f t="shared" ref="E35:E40" si="0">D35/C35</f>
         <v>0.4710009834294806</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="17" t="str">
+      <c r="A36" s="16" t="str">
         <f>A9</f>
         <v>INV/2026/06/002</v>
       </c>
-      <c r="B36" s="18">
+      <c r="B36" s="17">
         <f>G9</f>
         <v>2015.63</v>
       </c>
-      <c r="C36" s="19">
+      <c r="C36" s="18">
         <f>L9</f>
         <v>0</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="14">
         <f t="shared" ref="D36:D39" si="1">C36-B36</f>
         <v>-2015.63</v>
       </c>
-      <c r="E36" s="16" t="e">
+      <c r="E36" s="15" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="str">
+      <c r="A37" s="11" t="str">
         <f>A13</f>
         <v>INV/2026/06/003</v>
       </c>
-      <c r="B37" s="13">
+      <c r="B37" s="12">
         <f>G13</f>
         <v>6764.585</v>
       </c>
-      <c r="C37" s="14">
+      <c r="C37" s="13">
         <f>L13</f>
         <v>6561.68</v>
       </c>
-      <c r="D37" s="15">
+      <c r="D37" s="14">
         <f t="shared" si="1"/>
         <v>-202.90499999999975</v>
       </c>
-      <c r="E37" s="16">
+      <c r="E37" s="15">
         <f t="shared" si="0"/>
         <v>-3.0922721010472887E-2</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="17" t="str">
+      <c r="A38" s="16" t="str">
         <f>A18</f>
         <v>INV/2026/06/004</v>
       </c>
-      <c r="B38" s="18">
+      <c r="B38" s="17">
         <f>G18</f>
         <v>13529.16</v>
       </c>
-      <c r="C38" s="19">
+      <c r="C38" s="18">
         <f>L18</f>
         <v>13123.36</v>
       </c>
-      <c r="D38" s="15">
+      <c r="D38" s="14">
         <f t="shared" si="1"/>
         <v>-405.79999999999927</v>
       </c>
-      <c r="E38" s="16">
+      <c r="E38" s="15">
         <f t="shared" si="0"/>
         <v>-3.0921959010497255E-2</v>
       </c>
     </row>
     <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="str">
+      <c r="A39" s="11" t="str">
         <f>A24</f>
         <v>INV/2026/06/005</v>
       </c>
-      <c r="B39" s="13">
+      <c r="B39" s="12">
         <f>G24</f>
         <v>8309.5419999999995</v>
       </c>
-      <c r="C39" s="14">
+      <c r="C39" s="13">
         <f>L24</f>
         <v>2440.94</v>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="14">
         <f t="shared" si="1"/>
         <v>-5868.601999999999</v>
       </c>
-      <c r="E39" s="16">
+      <c r="E39" s="15">
         <f t="shared" si="0"/>
         <v>-2.4042385310577066</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A40" s="20" t="s">
+      <c r="A40" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B40" s="21">
+      <c r="B40" s="20">
         <f>SUM(B35:B39)</f>
         <v>41500.887000000002</v>
       </c>
-      <c r="C40" s="22">
+      <c r="C40" s="21">
         <f>SUM(C35:C39)</f>
         <v>42696.850000000006</v>
       </c>
-      <c r="D40" s="23">
+      <c r="D40" s="22">
         <f>SUM(D35:D39)</f>
         <v>1195.9630000000016</v>
       </c>
-      <c r="E40" s="24">
-        <f t="shared" si="0"/>
+      <c r="E40" s="23">
+        <f>D40/C40</f>
         <v>2.8010567524302178E-2</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A41" s="25" t="s">
+      <c r="A41" s="24" t="s">
         <v>44</v>
       </c>
-      <c r="B41" s="26">
+      <c r="B41" s="25">
         <f>SUM(F7,F11,F16,F22,F28)</f>
         <v>15287.715</v>
       </c>

</xml_diff>